<commit_message>
docs: add ステージ column to テスト仕様書 and update gen_testspec.ps1
</commit_message>
<xml_diff>
--- a/docs/テスト仕様書/テスト仕様書.xlsx
+++ b/docs/テスト仕様書/テスト仕様書.xlsx
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{646733E9-4B06-4F54-AF8C-C19A48C2627A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9C0632-04FB-4FBF-A641-0ACCDAE82BCF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9C0632-04FB-4FBF-A641-0ACCDAE82BCF}" activeTab="-1"/>
   </bookViews>
   <sheets>
-    <sheet name="テスト仕様書" sheetId="1" r:id="rId1"/>
+    <sheet name="テスト仕様書" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,12 +34,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>テスト区分</t>
+    <t>ステージ</t>
+  </si>
+  <si>
+    <t>テスト種別</t>
   </si>
   <si>
     <t>テスト項目</t>
@@ -48,23 +51,383 @@
     <t>操作手順</t>
   </si>
   <si>
-    <t>期待結果</t>
-  </si>
-  <si>
-    <t>合否</t>
+    <t>確認内容</t>
+  </si>
+  <si>
+    <t>期待される挙動</t>
+  </si>
+  <si>
+    <t>優先度</t>
+  </si>
+  <si>
+    <t>正常系</t>
+  </si>
+  <si>
+    <t>収支追加</t>
+  </si>
+  <si>
+    <t>支出レコードを追加できる</t>
+  </si>
+  <si>
+    <t>FAB(＋)をクリック→支出・食費・1000・2026-04-01 入力→追加</t>
+  </si>
+  <si>
+    <t>一覧に追加したレコードが表示される</t>
+  </si>
+  <si>
+    <t>食費 1000円のカードが一覧に表示される</t>
+  </si>
+  <si>
+    <t>高</t>
+  </si>
+  <si>
+    <t>収入レコードを追加できる</t>
+  </si>
+  <si>
+    <t>FAB(＋)→収入・給与・300000・2026-04-01→追加</t>
+  </si>
+  <si>
+    <t>一覧に収入レコードが追加される</t>
+  </si>
+  <si>
+    <t>給与 +¥300,000 が緑色で表示される</t>
+  </si>
+  <si>
+    <t>メモ付きで追加できる</t>
+  </si>
+  <si>
+    <t>FAB(＋)→支出・娯楽・5000・メモ「映画」→追加</t>
+  </si>
+  <si>
+    <t>メモが一覧に表示される</t>
+  </si>
+  <si>
+    <t>カード内に「映画」のメモが表示される</t>
+  </si>
+  <si>
+    <t>中</t>
+  </si>
+  <si>
+    <t>異常系</t>
+  </si>
+  <si>
+    <t>金額 0 は追加できない</t>
+  </si>
+  <si>
+    <t>FAB(＋)→支出・食費・0→追加</t>
+  </si>
+  <si>
+    <t>エラーメッセージが表示される</t>
+  </si>
+  <si>
+    <t>「入力値を確認してください」が赤字で表示され追加されない</t>
+  </si>
+  <si>
+    <t>金額が小数は追加できない</t>
+  </si>
+  <si>
+    <t>FAB(＋)→支出・食費・100.5→追加</t>
+  </si>
+  <si>
+    <t>金額が空は追加できない</t>
+  </si>
+  <si>
+    <t>FAB(＋)→支出・食費・(空)→追加</t>
+  </si>
+  <si>
+    <t>日付は当日がデフォルト設定される</t>
+  </si>
+  <si>
+    <t>FAB(＋)をクリックして日付フィールドを確認</t>
+  </si>
+  <si>
+    <t>日付フィールドに当日の日付が設定されている</t>
+  </si>
+  <si>
+    <t>システム日付と同じ値が入力済みになっている</t>
+  </si>
+  <si>
+    <t>種別切替でカテゴリが変わる</t>
+  </si>
+  <si>
+    <t>FAB(＋)→収入を選択してカテゴリ選択肢を確認</t>
+  </si>
+  <si>
+    <t>カテゴリに収入カテゴリが表示される</t>
+  </si>
+  <si>
+    <t>給与・ボーナス・副収入・投資・その他収入が表示される</t>
+  </si>
+  <si>
+    <t>収支編集</t>
+  </si>
+  <si>
+    <t>レコードを編集できる</t>
+  </si>
+  <si>
+    <t>一覧のレコードをクリック→金額を 2000 に変更→更新</t>
+  </si>
+  <si>
+    <t>一覧の金額が更新される</t>
+  </si>
+  <si>
+    <t>対象カードの金額が¥2,000 に変更されている</t>
+  </si>
+  <si>
+    <t>カテゴリを編集できる</t>
+  </si>
+  <si>
+    <t>一覧のレコードをクリック→カテゴリを「交通費」に変更→更新</t>
+  </si>
+  <si>
+    <t>一覧のカテゴリが更新される</t>
+  </si>
+  <si>
+    <t>対象カードのカテゴリが「交通費」に変更されている</t>
+  </si>
+  <si>
+    <t>編集モーダルに既存値が設定される</t>
+  </si>
+  <si>
+    <t>既存レコードをクリックしてフォームを確認</t>
+  </si>
+  <si>
+    <t>各フィールドに保存済みの値が入っている</t>
+  </si>
+  <si>
+    <t>日付・種別・カテゴリ・金額・メモが元の値で表示される</t>
+  </si>
+  <si>
+    <t>編集モードに削除ボタンが表示される</t>
+  </si>
+  <si>
+    <t>既存レコードをクリックしてモーダルを確認</t>
+  </si>
+  <si>
+    <t>「削除」ボタンが表示されている</t>
+  </si>
+  <si>
+    <t>追加モードでは非表示、編集モードでは表示される</t>
+  </si>
+  <si>
+    <t>収支削除</t>
+  </si>
+  <si>
+    <t>レコードを削除できる</t>
+  </si>
+  <si>
+    <t>既存レコードをクリック→削除→確認ダイアログで OK</t>
+  </si>
+  <si>
+    <t>一覧から対象レコードが消える</t>
+  </si>
+  <si>
+    <t>削除したカードが一覧から除去され、サマリーも更新される</t>
+  </si>
+  <si>
+    <t>削除確認ダイアログでキャンセルは操作されない</t>
+  </si>
+  <si>
+    <t>削除→確認ダイアログでキャンセル</t>
+  </si>
+  <si>
+    <t>レコードが削除されない</t>
+  </si>
+  <si>
+    <t>一覧に元のレコードがそのまま残る</t>
+  </si>
+  <si>
+    <t>全レコード削除後は空メッセージが表示される</t>
+  </si>
+  <si>
+    <t>当月の全レコードを削除</t>
+  </si>
+  <si>
+    <t>「記録がありません」が表示される</t>
+  </si>
+  <si>
+    <t>空メッセージが表示される</t>
+  </si>
+  <si>
+    <t>月ナビゲーション</t>
+  </si>
+  <si>
+    <t>前月ボタンで前月に切り替わる</t>
+  </si>
+  <si>
+    <t>ヘッダーの ‹ ボタンをクリック</t>
+  </si>
+  <si>
+    <t>ヘッダーの月表示が前月になる</t>
+  </si>
+  <si>
+    <t>例：2026年4月 → 2026年3月 に変わる</t>
+  </si>
+  <si>
+    <t>翌月ボタンで翌月に切り替わる</t>
+  </si>
+  <si>
+    <t>ヘッダーの › ボタンをクリック</t>
+  </si>
+  <si>
+    <t>ヘッダーの月表示が翌月になる</t>
+  </si>
+  <si>
+    <t>例：2026年4月 → 2026年5月 に変わる</t>
+  </si>
+  <si>
+    <t>別月のレコードは表示されない</t>
+  </si>
+  <si>
+    <t>5月にレコードを追加後、ヘッダーで4月に戻る</t>
+  </si>
+  <si>
+    <t>4月の一覧に5月のレコードが表示されない</t>
+  </si>
+  <si>
+    <t>月ごとにデータがフィルタリングされている</t>
+  </si>
+  <si>
+    <t>年をまたぐ月切替ができる</t>
+  </si>
+  <si>
+    <t>1月表示で ‹ ボタンをクリック</t>
+  </si>
+  <si>
+    <t>前年12月に切り替わる</t>
+  </si>
+  <si>
+    <t>例：2026年1月 → 2025年12月 に変わる</t>
+  </si>
+  <si>
+    <t>サマリー計算</t>
+  </si>
+  <si>
+    <t>収入合計が正しく計算される</t>
+  </si>
+  <si>
+    <t>給与30万・副収入5万を追加してサマリーを確認</t>
+  </si>
+  <si>
+    <t>収入カードに¥350,000 が表示される</t>
+  </si>
+  <si>
+    <t>すべての収入レコードの合計が表示される</t>
+  </si>
+  <si>
+    <t>支出合計が正しく計算される</t>
+  </si>
+  <si>
+    <t>食費1万・交通費3千を追加してサマリーを確認</t>
+  </si>
+  <si>
+    <t>支出カードに¥13,000 が表示される</t>
+  </si>
+  <si>
+    <t>すべての支出レコードの合計が表示される</t>
+  </si>
+  <si>
+    <t>残高が正しく計算される</t>
+  </si>
+  <si>
+    <t>収入20万・支出5万を追加してサマリーを確認</t>
+  </si>
+  <si>
+    <t>残高カードに¥150,000 が表示される</t>
+  </si>
+  <si>
+    <t>収入 − 支出 が正しく表示される</t>
+  </si>
+  <si>
+    <t>残高がマイナスの場合も表示される</t>
+  </si>
+  <si>
+    <t>支出のみ追加してサマリーを確認</t>
+  </si>
+  <si>
+    <t>残高カードに負の金額が表示される</t>
+  </si>
+  <si>
+    <t>¥-10,000 のように負の値が正しく表示される</t>
+  </si>
+  <si>
+    <t>チャート表示</t>
+  </si>
+  <si>
+    <t>支出カテゴリのチャートが表示される</t>
+  </si>
+  <si>
+    <t>複数カテゴリの支出を追加してチャートを確認</t>
+  </si>
+  <si>
+    <t>ドーナツチャートが描画される</t>
+  </si>
+  <si>
+    <t>カテゴリ別のチャートと凡例が表示される</t>
+  </si>
+  <si>
+    <t>支出がない場合は空メッセージを表示</t>
+  </si>
+  <si>
+    <t>収入のみ追加してチャートを確認</t>
+  </si>
+  <si>
+    <t>「支出データがありません」が表示される</t>
+  </si>
+  <si>
+    <t>チャートは非表示になり、テキストが表示される</t>
+  </si>
+  <si>
+    <t>月切替でチャートが更新される</t>
+  </si>
+  <si>
+    <t>別月に切り替えてチャートを確認</t>
+  </si>
+  <si>
+    <t>切替後の月の支出で再描画される</t>
+  </si>
+  <si>
+    <t>前月のデータではなく当月のデータが反映される</t>
+  </si>
+  <si>
+    <t>CSV出力</t>
+  </si>
+  <si>
+    <t>当月レコードを CSV でダウンロードできる</t>
+  </si>
+  <si>
+    <t>レコードを追加後、「CSV出力」ボタンをクリック</t>
+  </si>
+  <si>
+    <t>CSV ファイルがダウンロードされる</t>
+  </si>
+  <si>
+    <t>moneybook_2026-04.csv がダウンロードされる</t>
+  </si>
+  <si>
+    <t>CSV のヘッダー行が正しい</t>
+  </si>
+  <si>
+    <t>ダウンロードした CSV をテキストエディタで確認</t>
+  </si>
+  <si>
+    <t>1行目がヘッダー行になっている</t>
+  </si>
+  <si>
+    <t>「日付,種別,カテゴリ,金額,メモ」の順で記載される</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="游ゴシック"/>
       <family val="2"/>
-      <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -72,30 +435,16 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="游ゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <name val="游ゴシック"/>
       <family val="2"/>
-      <charset val="128"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="22"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -112,12 +461,21 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -134,6 +492,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TestSpec" displayName="TestSpec" ref="A1:H29" headerRowCount="1">
+  <autoFilter ref="A1:H29"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="No"/>
+    <tableColumn id="2" name="ステージ"/>
+    <tableColumn id="3" name="テスト種別"/>
+    <tableColumn id="4" name="テスト項目"/>
+    <tableColumn id="5" name="操作手順"/>
+    <tableColumn id="6" name="確認内容"/>
+    <tableColumn id="7" name="期待される挙動"/>
+    <tableColumn id="8" name="優先度"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -432,38 +807,778 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E153C9F8-1893-4D73-BB20-03ABAB9AEB15}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.8984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6" customWidth="1" style="2"/>
+    <col min="2" max="2" width="12" customWidth="1" style="2"/>
+    <col min="3" max="3" width="18" customWidth="1" style="2"/>
+    <col min="4" max="4" width="36" customWidth="1" style="2"/>
+    <col min="5" max="5" width="46" customWidth="1" style="2"/>
+    <col min="6" max="6" width="36" customWidth="1" style="2"/>
+    <col min="7" max="7" width="46" customWidth="1" style="2"/>
+    <col min="8" max="8" width="10" customWidth="1" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>